<commit_message>
Unify garden data source: read capacity from gardens.json
- Add capacity field to all gardens in gardens.json (value: 3)
- Update build_gardens_dataframe_from_json to read capacity from JSON
- Replace ensure_gardens_input_file with a direct JSON read — eliminates Gardens_Matching_Input.xlsx dependency
- Move Gardens_Matching_Input.xlsx to _archive (no longer needed)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Gale_Shapley_Matching_Result.xlsx
+++ b/Gale_Shapley_Matching_Result.xlsx
@@ -482,7 +482,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>גן דרקונצ'יק</t>
+          <t>משפחתון השקדיה</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -492,12 +492,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>תל חי 47</t>
+          <t>טרומן 33</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 3</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>גן אמנויות נילי</t>
+          <t>גן גפן</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -534,7 +534,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>תל חי 68</t>
+          <t>דבורה הנביאה 12</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -650,17 +650,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>הבית של אורה</t>
+          <t>הגן של רבקה</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>שכונת רמת שקמה</t>
+          <t>שכונת נחלת גנים</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>בניהו 18</t>
+          <t>האם 20</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -692,17 +692,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>הבית של רינת</t>
+          <t>גן דרקונצ'יק</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>שכונת תל בנימין</t>
+          <t>שכונת מתחם נגבה</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>תל חי 68</t>
+          <t>תל חי 47</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -776,22 +776,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>גן תותי</t>
+          <t>הבית של רינת</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>שכונת מתחם נגבה</t>
+          <t>שכונת תל בנימין</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>חד נס 33</t>
+          <t>תל חי 68</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>משפחתון השקדיה</t>
+          <t>הגן של רבקה</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>טרומן 33</t>
+          <t>החי"ל 32</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>הגן של רמי יעלים</t>
+          <t>גן כוכב</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -912,12 +912,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>החי"ל 38</t>
+          <t>שד הצנחנים 18</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>עדיפות 3</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -1112,17 +1112,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>המשפחתון של אולה</t>
+          <t>הבית של רינת</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>שכונת שיכון ותיקים</t>
+          <t>שכונת תל בנימין</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>בועז 6</t>
+          <t>תל חי 68</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1154,17 +1154,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>יהדות בחוויה</t>
+          <t>הקטנטנים של אורלי</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>שכונת איצטדיון</t>
+          <t>שכונת רמת שקמה</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>רוקח 121</t>
+          <t>שמעוני 5</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1364,17 +1364,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>יהדות בחוויה</t>
+          <t>גן פורח</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>שכונת איצטדיון</t>
+          <t>שכונת גפן</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>רוקח 121</t>
+          <t>רוקח 37</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1406,17 +1406,17 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>מיכאלה</t>
+          <t>הגן של אביה</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>שכונת תל יהודה</t>
+          <t>שכונת תל גנים</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>אהוד 4</t>
+          <t>גדעון 30</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>גן פורח</t>
+          <t>הפינוקייה</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1500,12 +1500,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>רוקח 37</t>
+          <t>דרך אבא הלל 110</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -1532,17 +1532,17 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>גן פורח</t>
+          <t>יהדות בחוויה</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>שכונת גפן</t>
+          <t>שכונת איצטדיון</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>רוקח 37</t>
+          <t>רוקח 121</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1616,22 +1616,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>גן טניהלנד</t>
+          <t>גן פורח</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>שכונת רמת חן</t>
+          <t>שכונת גפן</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>קרייתי 6</t>
+          <t>רוקח 37</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -1742,17 +1742,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>גן שרה</t>
+          <t>רוני רון</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>שכונת רמת עמידר</t>
+          <t>שכונת אזור הבילויים</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>דרך התפוצות 84</t>
+          <t>דיין משה 19</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1784,17 +1784,17 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>משפחתון בובליק</t>
+          <t>פשוש תל השומר</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>שכונת אזור הבילויים</t>
+          <t>שכונת תל השומר</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>שד הקונגרס 17</t>
+          <t>עמק דותן 24</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1826,17 +1826,17 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>גן מורן ברקוביץ</t>
+          <t>משפחתון בובליק</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>שכונת חרוזים</t>
+          <t>שכונת אזור הבילויים</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>המלאכה 14</t>
+          <t>שד הקונגרס 17</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>גן מדינת הילדים</t>
+          <t>רוני רון</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>נטר 12</t>
+          <t>דיין משה 19</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1952,7 +1952,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>גן מאלף עד טף</t>
+          <t>דומיק</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1962,12 +1962,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>הרא"ה 287</t>
+          <t>שד הקונגרס 6</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -2078,22 +2078,22 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>גן קטנטנים</t>
+          <t>יהדות בחוויה</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>שכונת אזור הבילויים</t>
+          <t>שכונת איצטדיון</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>אבן ספיר 6</t>
+          <t>רוקח 121</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -2120,17 +2120,17 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>פנדה גן</t>
+          <t>גן מדינת הילדים</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>שכונת תל יהודה</t>
+          <t>שכונת אזור הבילויים</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>אלרואי 12</t>
+          <t>נטר 12</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2288,17 +2288,17 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>פשוש תל השומר</t>
+          <t>המשפחתון של עדינה</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>שכונת תל השומר</t>
+          <t>שכונת גפן</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>עמק דותן 24</t>
+          <t>המתמיד 20</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2330,17 +2330,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>פני פרלמן</t>
+          <t>משפחתון חיפושית</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>שכונת שיכון ותיקים</t>
+          <t>שכונת רמת עמידר</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>שד הנרקיסים 31</t>
+          <t>דרך התפוצות 40</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>גן לאה</t>
+          <t>מעון רא"ם</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2382,12 +2382,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>קוממיות 3</t>
+          <t>חמיר 6</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>עדיפות 3</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>המשפחתון של סילביה</t>
+          <t>גן שרה</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2424,7 +2424,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>המעפיל 14</t>
+          <t>דרך התפוצות 84</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2456,17 +2456,17 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>גן לאה</t>
+          <t>גן סאנשיין</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>שכונת רמת עמידר</t>
+          <t>שכונת נווה יהושע</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>קוממיות 3</t>
+          <t>בן אליעזר אריה 38</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2498,17 +2498,17 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>מעון רא"ם</t>
+          <t>הממלכה של סילבי</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>שכונת רמת עמידר</t>
+          <t>שכונת מתחם נגבה</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>חמיר 6</t>
+          <t>תל חי 68</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2582,17 +2582,17 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>גן טיף טף  הגן של עדנה</t>
+          <t>מעון רא"ם</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>שכונת נווה יהושע</t>
+          <t>שכונת רמת עמידר</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>נוה יהושע 19</t>
+          <t>חמיר 6</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>המשפחתון של אולה</t>
+          <t>גן מעון הנרקיסים</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>בועז 6</t>
+          <t>שד הנרקיסים 50</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -3044,7 +3044,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>גן ילדים בייבי קונסרבטוריון</t>
+          <t>גן בייביקט</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3054,12 +3054,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>בר כוכבא 28</t>
+          <t>מוצא 8</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>גן ילדים בייבי קונסרבטוריון</t>
+          <t>גן בייביקט</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3138,12 +3138,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>בר כוכבא 28</t>
+          <t>מוצא 8</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -3170,7 +3170,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>האפי לנד</t>
+          <t>גן ילדים בייבי קונסרבטוריון</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3180,12 +3180,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>הרא"ה 169</t>
+          <t>בר כוכבא 28</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>גן ישראל  חינוך מאיר</t>
+          <t>האפי לנד</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3222,12 +3222,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>מוצא 7</t>
+          <t>הרא"ה 169</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -3254,7 +3254,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>גן קטקטים</t>
+          <t>גן קשת מונטסורי</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>מאיר בעל הנס 13</t>
+          <t>כנפי נשרים 12</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>התמרים</t>
+          <t>הפצפונים של זיוה</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3306,12 +3306,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>שד התמרים 4</t>
+          <t>שד התמרים 10</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -3380,7 +3380,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>עם יעלי</t>
+          <t>התמרים</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3390,12 +3390,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>שרת משה 19</t>
+          <t>שד התמרים 4</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -3422,17 +3422,17 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>גן גוונים</t>
+          <t>גן שורשים</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>שכונת בן גוריון</t>
+          <t>שכונת גפן</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>קריניצי 67</t>
+          <t>ברנשטיין פרץ 42</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>חושחושים</t>
+          <t>הפצפונים של זיוה</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3474,12 +3474,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>השר משה 45</t>
+          <t>שד התמרים 10</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -3506,7 +3506,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>הפצפונים של זיוה</t>
+          <t>חושחושים</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3516,7 +3516,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>שד התמרים 10</t>
+          <t>השר משה 45</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3926,7 +3926,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>רמת שקמה ב</t>
+          <t>בייבי קונסרבטוריון</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3936,12 +3936,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>אחד העם 18</t>
+          <t>שמעוני 10</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -4094,7 +4094,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>שד ויצו שקמה ג</t>
+          <t>רמת שקמה ב</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -4104,12 +4104,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>אחד העם 59</t>
+          <t>אחד העם 18</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -4388,17 +4388,17 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>קרני ראם</t>
+          <t>משפחתון טינקי</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>שכונת רמת עמידר</t>
+          <t>שכונת רמת חן</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>מבצע עין 9</t>
+          <t>שד בן צבי 3</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -4430,7 +4430,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>גן בתנועה</t>
+          <t>פני פרלמן</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>רוקח 102</t>
+          <t>שד הנרקיסים 31</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -4724,17 +4724,17 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>ריינבו</t>
+          <t>קרני ראם</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>שכונת מרכז העיר</t>
+          <t>שכונת רמת עמידר</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>ביאליק 37</t>
+          <t>מבצע עין 9</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -4850,17 +4850,17 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>גן רון לי</t>
+          <t>המשפחתון של שרון</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>שכונת הלל</t>
+          <t>שכונת גפן</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>הגלגל 20</t>
+          <t>צוריאל 6</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -4892,17 +4892,17 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>המשפחתון של עדינה</t>
+          <t>גן מורן ברקוביץ</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>שכונת גפן</t>
+          <t>שכונת חרוזים</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>המתמיד 20</t>
+          <t>המלאכה 14</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -5060,22 +5060,22 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>גן סאנשיין</t>
+          <t>ביהייב פליי סקול</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>שכונת נווה יהושע</t>
+          <t>שכונת חשמונאים</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>בן אליעזר אריה 38</t>
+          <t>השוטרת 14</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 3</t>
         </is>
       </c>
     </row>
@@ -5144,7 +5144,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>גן כוכב</t>
+          <t>עולם קטן</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -5154,12 +5154,12 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>סמ המעלות 4</t>
+          <t>בעל שם טוב 13</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5186,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>גן צוף</t>
+          <t>מסיבת גן אצל תמי</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -5196,12 +5196,12 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>מרים 11</t>
+          <t>המעגל 12</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -5228,7 +5228,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>מסיבת גן אצל תמי</t>
+          <t>גן צוף</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -5238,12 +5238,12 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>המעגל 12</t>
+          <t>מרים 11</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -5354,7 +5354,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>הקטקטים של עדית</t>
+          <t>אכא עמותה לקידום חינוך הוליסטי</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -5364,12 +5364,12 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>אלונים 9</t>
+          <t>ויינשל אליעזר 4</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -5480,17 +5480,17 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>גן שורשים</t>
+          <t>גן ישראל חינוך מאיר</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>שכונת גפן</t>
+          <t>שכונת קריית בורוכוב</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>ברנשטיין פרץ 42</t>
+          <t>גרנדוס 35</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -5732,7 +5732,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>גן מרים</t>
+          <t>גן אמנויות נילי</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -5742,12 +5742,12 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>ישורון 13</t>
+          <t>תפארת ישראל 5</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -6278,17 +6278,17 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>גן שורשים</t>
+          <t>קרני ראם</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>שכונת גפן</t>
+          <t>שכונת רמת עמידר</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>ברנשטיין פרץ 42</t>
+          <t>מבצע עין 9</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -6320,17 +6320,17 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>גן בצוללת צהובה</t>
+          <t>אכא עמותה לקידום חינוך הוליסטי</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>שכונת נחלת גנים</t>
+          <t>שכונת הלל</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>העמל 15</t>
+          <t>הגלגל 55</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -6824,22 +6824,22 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>גן קשת</t>
+          <t>גן מיכאלה שיכון ותיקים</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>שכונת מרכז העיר</t>
+          <t>שכונת שיכון ותיקים</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>הרצל 49</t>
+          <t>יעלים 2</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>עדיפות 3</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -6866,17 +6866,17 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>המשפחתון של שרון</t>
+          <t>גן רון לי</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>שכונת גפן</t>
+          <t>שכונת הלל</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>צוריאל 6</t>
+          <t>הגלגל 20</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
@@ -6992,22 +6992,22 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>גן ישראל חינוך מאיר</t>
+          <t>מיכאלה</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>שכונת קריית בורוכוב</t>
+          <t>שכונת תל יהודה</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>גרנדוס 35</t>
+          <t>אהוד 5</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 3</t>
         </is>
       </c>
     </row>
@@ -7160,7 +7160,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>גן מאלף עד טף</t>
+          <t>משפחתון בובליק</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -7170,12 +7170,12 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>הרא"ה 287</t>
+          <t>שד הקונגרס 17</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -7412,22 +7412,22 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>גן צמרת | גן צמרת  התינוקיה</t>
+          <t>גן קטנטנים</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>שכונת עליות</t>
+          <t>שכונת אזור הבילויים</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>האגדה 16</t>
+          <t>אבן ספיר 6</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -7496,7 +7496,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>לאמה גן</t>
+          <t>הבית של עינבי</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -7506,12 +7506,12 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>דרך בן גוריון דוד 117</t>
+          <t>ביאליק 123</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 3</t>
         </is>
       </c>
     </row>
@@ -7832,7 +7832,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>מעון רא"ם</t>
+          <t>הגן של יפה</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -7842,12 +7842,12 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>חמיר 6</t>
+          <t>בן אליעזר אריה 29</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -7916,7 +7916,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>גן גפן</t>
+          <t>גן תותי</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -7926,12 +7926,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>דבורה הנביאה 12</t>
+          <t>חד נס 33</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -8000,7 +8000,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>גן בייביקט</t>
+          <t>גן ישראל  חינוך מאיר</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -8010,12 +8010,12 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>מוצא 8</t>
+          <t>מוצא 7</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -8084,7 +8084,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>גן מעון הנרקיסים</t>
+          <t>המשפחתון של אולה</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>שד הנרקיסים 50</t>
+          <t>בועז 6</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
@@ -8294,7 +8294,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>הבית של יעל</t>
+          <t>גן אמנויות נילי</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -8304,12 +8304,12 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>מוריה 38</t>
+          <t>תפארת ישראל 5</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>עדיפות 3</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -8378,7 +8378,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>גן כוכב</t>
+          <t>גן צוף</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -8388,12 +8388,12 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>סמ המעלות 4</t>
+          <t>מרים 11</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -8462,22 +8462,22 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>רוני רון</t>
+          <t>גן בצוללת צהובה</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>שכונת אזור הבילויים</t>
+          <t>שכונת נחלת גנים</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>דיין משה 19</t>
+          <t>העמל 15</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -8546,17 +8546,17 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>האפרוחים של איילת</t>
+          <t>ריינבו</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>שכונת יד לבנים</t>
+          <t>שכונת מרכז העיר</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>חיבת ציון 10</t>
+          <t>ביאליק 37</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
@@ -8588,22 +8588,22 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>גן הבית של אמא</t>
+          <t>גן קטקטים</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>שכונת אזור הבילויים</t>
+          <t>שכונת מרום נווה</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>דיין משה 13</t>
+          <t>מאיר בעל הנס 13</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>עדיפות 3</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -8714,17 +8714,17 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>הבית של עינבי</t>
+          <t>גן פורח</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>שכונת שיכון ותיקים</t>
+          <t>שכונת גפן</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>בועז 14</t>
+          <t>רוקח 37</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
@@ -8756,7 +8756,7 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>הבית של רינת</t>
+          <t>הקטקטים של עדית</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
@@ -8766,12 +8766,12 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>תל חי 68</t>
+          <t>אלונים 9</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -8840,17 +8840,17 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>הקטנטנים של אורלי</t>
+          <t>הגן של מיכל ואורנה</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>שכונת רמת שקמה</t>
+          <t>שכונת רמת חן</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>שמעוני 5</t>
+          <t>אלוף דוד 59</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
@@ -9050,7 +9050,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>מעון רא"ם</t>
+          <t>גן לאה</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
@@ -9060,12 +9060,12 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>חמיר 6</t>
+          <t>קוממיות 3</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 3</t>
         </is>
       </c>
     </row>
@@ -9092,22 +9092,22 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>גן קשת מונטסורי</t>
+          <t>הגן של נתן</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>שכונת מרום נווה</t>
+          <t>שכונת נווה יהושע</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>כנפי נשרים 12</t>
+          <t>הררי 28</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -9176,7 +9176,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>מיכאלה</t>
+          <t>משפחתון מאירה</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
@@ -9186,12 +9186,12 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>אהוד 5</t>
+          <t>רוחמה 35</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -9302,7 +9302,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>משפחתון אירנה</t>
+          <t>גן שרה</t>
         </is>
       </c>
       <c r="F212" t="inlineStr">
@@ -9312,12 +9312,12 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>בן אליעזר אריה 10</t>
+          <t>דרך התפוצות 84</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -9344,22 +9344,22 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>רוני רון</t>
+          <t>הקטנטנים של אורלי</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>שכונת אזור הבילויים</t>
+          <t>שכונת רמת שקמה</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>דיין משה 19</t>
+          <t>שמעוני 5</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>עדיפות 3</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -9638,7 +9638,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>גן אמנויות נילי</t>
+          <t>גן מרים</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
@@ -9648,12 +9648,12 @@
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>תפארת ישראל 5</t>
+          <t>ישורון 13</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -9680,7 +9680,7 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>גן כוכב</t>
+          <t>הגן של רמי יעלים</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
@@ -9690,12 +9690,12 @@
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>שד הצנחנים 18</t>
+          <t>החי"ל 38</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -9764,7 +9764,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>אכא עמותה לקידום חינוך הוליסטי</t>
+          <t>לאמה גן</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
@@ -9774,12 +9774,12 @@
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>הגלגל 55</t>
+          <t>דרך בן גוריון דוד 117</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -9848,22 +9848,22 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>עולם קטן</t>
+          <t>הבית של עינבי</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>שכונת חשמונאים</t>
+          <t>שכונת שיכון ותיקים</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>בעל שם טוב 13</t>
+          <t>בועז 14</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -9932,22 +9932,22 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>הגן של יפה</t>
+          <t>גן קשת</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>שכונת רמת עמידר</t>
+          <t>שכונת מרכז העיר</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>בן אליעזר אריה 29</t>
+          <t>הרצל 49</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -9974,7 +9974,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>משפחתון חיפושית</t>
+          <t>גן לאה</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
@@ -9984,12 +9984,12 @@
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>דרך התפוצות 40</t>
+          <t>קוממיות 3</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -10058,7 +10058,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>גן פורח</t>
+          <t>גן שורשים</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
@@ -10068,7 +10068,7 @@
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>רוקח 37</t>
+          <t>ברנשטיין פרץ 42</t>
         </is>
       </c>
       <c r="H230" t="inlineStr">
@@ -10226,7 +10226,7 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>גן בייביקט</t>
+          <t>גן ילדים בייבי קונסרבטוריון</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
@@ -10236,12 +10236,12 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>מוצא 8</t>
+          <t>בר כוכבא 28</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -10310,7 +10310,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>משפחתון מאירה</t>
+          <t>פנדה קלאב</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
@@ -10320,12 +10320,12 @@
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>רוחמה 35</t>
+          <t>המלך יוסף 52</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -10352,7 +10352,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>גן קטנטנים</t>
+          <t>גן מדינת הילדים</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
@@ -10362,12 +10362,12 @@
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>אבן ספיר 6</t>
+          <t>נטר 12</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -10436,22 +10436,22 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>הגן של יפה</t>
+          <t>גן קשת</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>שכונת רמת עמידר</t>
+          <t>שכונת מרכז העיר</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>בן אליעזר אריה 29</t>
+          <t>הרצל 49</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -10478,22 +10478,22 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>גן פימפונים | פימפונים</t>
+          <t>הגן של יפה</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>שכונת נווה רם</t>
+          <t>שכונת רמת עמידר</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>פנקס 17</t>
+          <t>בן אליעזר אריה 29</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 3</t>
         </is>
       </c>
     </row>
@@ -10604,7 +10604,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>יהדות בחוויה</t>
+          <t>גן גוונים</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
@@ -10614,12 +10614,12 @@
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>קריניצי 70</t>
+          <t>קריניצי 67</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -10646,22 +10646,22 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>מהותי לא רק מעון יום</t>
+          <t>גן בגן</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>שכונת הבורסה</t>
+          <t>שכונת בן גוריון</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>יעקב רוזן 11</t>
+          <t>הרא"ה 11</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -10814,7 +10814,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>גן צוף</t>
+          <t>עולם קטן</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
@@ -10824,12 +10824,12 @@
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>מרים 11</t>
+          <t>בעל שם טוב 13</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 3</t>
         </is>
       </c>
     </row>
@@ -10898,7 +10898,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>גן נטלי</t>
+          <t>גן דרקונצ'יק</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
@@ -10908,12 +10908,12 @@
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t>חד נס 38</t>
+          <t>תל חי 47</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 3</t>
         </is>
       </c>
     </row>
@@ -10982,7 +10982,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>ביהייב פליי סקול</t>
+          <t>גן כוכב</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>השוטרת 14</t>
+          <t>הרב חבה אליה 3</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
@@ -11024,22 +11024,22 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>הממלכה של סילבי</t>
+          <t>מעון רא"ם</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>שכונת מתחם נגבה</t>
+          <t>שכונת רמת עמידר</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t>תל חי 68</t>
+          <t>חמיר 6</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -11150,22 +11150,22 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>משפחתון חיפושית</t>
+          <t>גן מאלף עד טף</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>שכונת רמת עמידר</t>
+          <t>שכונת אזור הבילויים</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t>דרך התפוצות 40</t>
+          <t>הרא"ה 287</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -11192,22 +11192,22 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>גן מדינת הילדים</t>
+          <t>גן טניהלנד</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>שכונת אזור הבילויים</t>
+          <t>שכונת רמת חן</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>נטר 12</t>
+          <t>קרייתי 6</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -11276,7 +11276,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>הגן של נתן</t>
+          <t>גן מונני</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
@@ -11286,12 +11286,12 @@
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>הררי 28</t>
+          <t>חבצלת 8</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -11570,17 +11570,17 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>אכא עמותה לקידום חינוך הוליסטי</t>
+          <t>גן פימפונים | פימפונים</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>שכונת תל בנימין</t>
+          <t>שכונת נווה רם</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>ויינשל אליעזר 4</t>
+          <t>פנקס 17</t>
         </is>
       </c>
       <c r="H266" t="inlineStr">
@@ -11780,7 +11780,7 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>דומיק</t>
+          <t>קן קטנטנים</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
@@ -11790,12 +11790,12 @@
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>שד הקונגרס 6</t>
+          <t>דיין משה 13</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -11864,17 +11864,17 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>שד ויצו שקמה ג</t>
+          <t>מהותי לא רק מעון יום</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>שכונת רמת שקמה</t>
+          <t>שכונת הבורסה</t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>אחד העם 59</t>
+          <t>יעקב רוזן 11</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">
@@ -11948,7 +11948,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>משפחתון אירנה</t>
+          <t>המשפחתון של סילביה</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
@@ -11958,12 +11958,12 @@
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>בן אליעזר אריה 10</t>
+          <t>המעפיל 14</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -11990,7 +11990,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>הגן של רבקה</t>
+          <t>גן דרקונצ'יק</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
@@ -12000,12 +12000,12 @@
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>החי"ל 32</t>
+          <t>תל חי 47</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -12074,7 +12074,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>עולם קטן</t>
+          <t>גן צוף</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
@@ -12084,12 +12084,12 @@
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>בעל שם טוב 13</t>
+          <t>מרים 11</t>
         </is>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 3</t>
         </is>
       </c>
     </row>
@@ -12116,22 +12116,22 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>לה קסיטה דה צ'וקולטה</t>
+          <t>גן כוכב</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>שכונת קריית בורוכוב</t>
+          <t>שכונת חשמונאים</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>עוזיאל 116</t>
+          <t>סמ המעלות 4</t>
         </is>
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -12326,7 +12326,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>משפחתון טינקי</t>
+          <t>גן הילדים</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -12336,12 +12336,12 @@
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>שד בן צבי 3</t>
+          <t>רזיאל 27</t>
         </is>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -12368,22 +12368,22 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>גן דרקונצ'יק</t>
+          <t>האפרוחים של איילת</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>שכונת מתחם נגבה</t>
+          <t>שכונת יד לבנים</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>תל חי 47</t>
+          <t>חיבת ציון 10</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -12620,7 +12620,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>גן מיכאלה שיכון ותיקים</t>
+          <t>המשפחתון של גלית</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
@@ -12630,12 +12630,12 @@
       </c>
       <c r="G291" t="inlineStr">
         <is>
-          <t>יעלים 2</t>
+          <t>רננים 14</t>
         </is>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -12746,7 +12746,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>גן דרקונצ'יק</t>
+          <t>גן נטלי</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
@@ -12756,12 +12756,12 @@
       </c>
       <c r="G294" t="inlineStr">
         <is>
-          <t>תל חי 47</t>
+          <t>חד נס 38</t>
         </is>
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -12872,7 +12872,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>המשפחתון של סילביה</t>
+          <t>משפחתון אירנה</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
@@ -12882,12 +12882,12 @@
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>המעפיל 14</t>
+          <t>בן אליעזר אריה 10</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 3</t>
         </is>
       </c>
     </row>
@@ -12998,7 +12998,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>הפצפונים של זיוה</t>
+          <t>עם יעלי</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
@@ -13008,12 +13008,12 @@
       </c>
       <c r="G300" t="inlineStr">
         <is>
-          <t>שד התמרים 10</t>
+          <t>שרת משה 19</t>
         </is>
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -13124,7 +13124,7 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>הילדים של אורטלי</t>
+          <t>גן תותי</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
@@ -13134,12 +13134,12 @@
       </c>
       <c r="G303" t="inlineStr">
         <is>
-          <t>טרומן 29</t>
+          <t>חד נס 33</t>
         </is>
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -13166,7 +13166,7 @@
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>קרני ראם</t>
+          <t>רמת עמידר</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
@@ -13176,12 +13176,12 @@
       </c>
       <c r="G304" t="inlineStr">
         <is>
-          <t>מבצע עין 9</t>
+          <t>דרך התפוצות 7</t>
         </is>
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -13208,7 +13208,7 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>רמת עמידר</t>
+          <t>המשפחתון של סילביה</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
@@ -13218,12 +13218,12 @@
       </c>
       <c r="G305" t="inlineStr">
         <is>
-          <t>דרך התפוצות 7</t>
+          <t>המעפיל 14</t>
         </is>
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 3</t>
         </is>
       </c>
     </row>
@@ -13250,7 +13250,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>גן כוכב</t>
+          <t>גן אמנויות נילי</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
@@ -13260,12 +13260,12 @@
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t>שד הצנחנים 18</t>
+          <t>תל חי 68</t>
         </is>
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>עדיפות 3</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -13292,22 +13292,22 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>גן הילדים</t>
+          <t>הממלכה של סילבי</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>שכונת רמת חן</t>
+          <t>שכונת מתחם נגבה</t>
         </is>
       </c>
       <c r="G307" t="inlineStr">
         <is>
-          <t>רזיאל 27</t>
+          <t>תל חי 68</t>
         </is>
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -13334,7 +13334,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>הממלכה של סילבי</t>
+          <t>גן כוכב</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
@@ -13344,12 +13344,12 @@
       </c>
       <c r="G308" t="inlineStr">
         <is>
-          <t>תל חי 68</t>
+          <t>שד הצנחנים 18</t>
         </is>
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -13502,22 +13502,22 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>גן כוכב</t>
+          <t>לה קסיטה דה צ'וקולטה</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>שכונת חשמונאים</t>
+          <t>שכונת קריית בורוכוב</t>
         </is>
       </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t>הרב חבה אליה 3</t>
+          <t>עוזיאל 116</t>
         </is>
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -13628,7 +13628,7 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>המשפחתון של גלית</t>
+          <t>גן בתנועה</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
@@ -13638,12 +13638,12 @@
       </c>
       <c r="G315" t="inlineStr">
         <is>
-          <t>רננים 14</t>
+          <t>רוקח 102</t>
         </is>
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -13754,7 +13754,7 @@
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>משפחתון מאירה</t>
+          <t>פנדה גן</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
@@ -13764,12 +13764,12 @@
       </c>
       <c r="G318" t="inlineStr">
         <is>
-          <t>רוחמה 35</t>
+          <t>אלרואי 12</t>
         </is>
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>עדיפות 3</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -13838,7 +13838,7 @@
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>גן תותי</t>
+          <t>גן נטלי</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
@@ -13848,12 +13848,12 @@
       </c>
       <c r="G320" t="inlineStr">
         <is>
-          <t>חד נס 33</t>
+          <t>חד נס 38</t>
         </is>
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -13922,7 +13922,7 @@
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>מסיבת גן אצל תמי</t>
+          <t>גן כוכב</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
@@ -13932,12 +13932,12 @@
       </c>
       <c r="G322" t="inlineStr">
         <is>
-          <t>המעגל 12</t>
+          <t>סמ המעלות 4</t>
         </is>
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 3</t>
         </is>
       </c>
     </row>
@@ -14300,17 +14300,17 @@
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>הפינוקייה</t>
+          <t>לה קסיטה דה צ'וקולטה</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>שכונת גפן</t>
+          <t>שכונת קריית בורוכוב</t>
         </is>
       </c>
       <c r="G331" t="inlineStr">
         <is>
-          <t>דרך אבא הלל 110</t>
+          <t>עוזיאל 116</t>
         </is>
       </c>
       <c r="H331" t="inlineStr">
@@ -14720,7 +14720,7 @@
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>גן שרה</t>
+          <t>משפחתון אירנה</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
@@ -14730,12 +14730,12 @@
       </c>
       <c r="G341" t="inlineStr">
         <is>
-          <t>דרך התפוצות 84</t>
+          <t>בן אליעזר אריה 10</t>
         </is>
       </c>
       <c r="H341" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -14762,22 +14762,22 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>הקטנטנים של אורלי</t>
+          <t>גן קטנטנים</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>שכונת רמת שקמה</t>
+          <t>שכונת אזור הבילויים</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>שמעוני 5</t>
+          <t>אבן ספיר 6</t>
         </is>
       </c>
       <c r="H342" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -14888,7 +14888,7 @@
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>קן קטנטנים</t>
+          <t>גן הבית של אמא</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
@@ -14903,7 +14903,7 @@
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -14930,17 +14930,17 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>הגן של מיכל ואורנה</t>
+          <t>גן צמרת | גן צמרת  התינוקיה</t>
         </is>
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>שכונת רמת חן</t>
+          <t>שכונת עליות</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t>אלוף דוד 59</t>
+          <t>האגדה 16</t>
         </is>
       </c>
       <c r="H346" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>פנדה קלאב</t>
+          <t>מיכאלה</t>
         </is>
       </c>
       <c r="F347" t="inlineStr">
@@ -14982,12 +14982,12 @@
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t>המלך יוסף 52</t>
+          <t>אהוד 4</t>
         </is>
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -15014,7 +15014,7 @@
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>הגן של יפה</t>
+          <t>משפחתון חיפושית</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
@@ -15024,12 +15024,12 @@
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t>בן אליעזר אריה 29</t>
+          <t>דרך התפוצות 40</t>
         </is>
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -15140,7 +15140,7 @@
       </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>גן בגן</t>
+          <t>יהדות בחוויה</t>
         </is>
       </c>
       <c r="F351" t="inlineStr">
@@ -15150,12 +15150,12 @@
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t>הרא"ה 11</t>
+          <t>קריניצי 70</t>
         </is>
       </c>
       <c r="H351" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -15224,22 +15224,22 @@
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>הבית של עינבי</t>
+          <t>גן מעון הנרקיסים</t>
         </is>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>שכונת הלל</t>
+          <t>שכונת שיכון ותיקים</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t>ביאליק 123</t>
+          <t>שד הנרקיסים 50</t>
         </is>
       </c>
       <c r="H353" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>מחוץ לרשימה</t>
         </is>
       </c>
     </row>
@@ -15392,7 +15392,7 @@
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>גן אמנויות נילי</t>
+          <t>הבית של יעל</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
@@ -15402,12 +15402,12 @@
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t>תפארת ישראל 5</t>
+          <t>מוריה 38</t>
         </is>
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -15728,7 +15728,7 @@
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t>גן מעון הנרקיסים</t>
+          <t>המשפחתון של אולה</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
@@ -15738,7 +15738,7 @@
       </c>
       <c r="G365" t="inlineStr">
         <is>
-          <t>שד הנרקיסים 50</t>
+          <t>בועז 6</t>
         </is>
       </c>
       <c r="H365" t="inlineStr">
@@ -15896,7 +15896,7 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>משפחתון בובליק</t>
+          <t>גן מאלף עד טף</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
@@ -15906,12 +15906,12 @@
       </c>
       <c r="G369" t="inlineStr">
         <is>
-          <t>שד הקונגרס 17</t>
+          <t>הרא"ה 287</t>
         </is>
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>עדיפות 3</t>
+          <t>עדיפות 1</t>
         </is>
       </c>
     </row>
@@ -15980,22 +15980,22 @@
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>גן קשת</t>
+          <t>הגן של יפה</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>שכונת מרכז העיר</t>
+          <t>שכונת רמת עמידר</t>
         </is>
       </c>
       <c r="G371" t="inlineStr">
         <is>
-          <t>הרצל 49</t>
+          <t>בן אליעזר אריה 29</t>
         </is>
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>מחוץ לרשימה</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -16022,7 +16022,7 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>גן מונני</t>
+          <t>גן טיף טף  הגן של עדנה</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
@@ -16032,12 +16032,12 @@
       </c>
       <c r="G372" t="inlineStr">
         <is>
-          <t>חבצלת 8</t>
+          <t>נוה יהושע 19</t>
         </is>
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -16148,7 +16148,7 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>בייבי קונסרבטוריון</t>
+          <t>הבית של אורה</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
@@ -16158,12 +16158,12 @@
       </c>
       <c r="G375" t="inlineStr">
         <is>
-          <t>שמעוני 10</t>
+          <t>בניהו 18</t>
         </is>
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 3</t>
         </is>
       </c>
     </row>
@@ -16274,7 +16274,7 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>גן צוף</t>
+          <t>מסיבת גן אצל תמי</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
@@ -16284,12 +16284,12 @@
       </c>
       <c r="G378" t="inlineStr">
         <is>
-          <t>מרים 11</t>
+          <t>המעגל 12</t>
         </is>
       </c>
       <c r="H378" t="inlineStr">
         <is>
-          <t>עדיפות 2</t>
+          <t>עדיפות 3</t>
         </is>
       </c>
     </row>
@@ -16316,7 +16316,7 @@
       </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t>גן נטלי</t>
+          <t>הילדים של אורטלי</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
@@ -16326,12 +16326,12 @@
       </c>
       <c r="G379" t="inlineStr">
         <is>
-          <t>חד נס 38</t>
+          <t>טרומן 29</t>
         </is>
       </c>
       <c r="H379" t="inlineStr">
         <is>
-          <t>עדיפות 1</t>
+          <t>עדיפות 2</t>
         </is>
       </c>
     </row>
@@ -16756,12 +16756,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>שד ויצו שקמה ג</t>
+          <t>הקטקטים של עדית</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>שכונת רמת שקמה</t>
+          <t>שכונת תל בנימין</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -16774,18 +16774,18 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>הקטקטים של עדית</t>
+          <t>פנדה גן</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>שכונת תל בנימין</t>
+          <t>שכונת תל יהודה</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -16798,7 +16798,7 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -16828,12 +16828,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>פנדה גן</t>
+          <t>הפעוטות של מירה</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>שכונת תל יהודה</t>
+          <t>שכונת ראשונים</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -16846,18 +16846,18 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>הפעוטות של מירה</t>
+          <t>בית קנדה קשת</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>שכונת ראשונים</t>
+          <t>שכונת נווה יהושע</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -16870,18 +16870,18 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>בית קנדה קשת</t>
+          <t>ריינבו</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>שכונת נווה יהושע</t>
+          <t>שכונת מרכז העיר</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -16894,7 +16894,7 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -16972,12 +16972,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ריינבו</t>
+          <t>הגן של יפה</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>שכונת מרכז העיר</t>
+          <t>שכונת רמת עמידר</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -16990,7 +16990,7 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
@@ -17020,12 +17020,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>הגן של יפה</t>
+          <t>גן סאנשיין</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>שכונת רמת עמידר</t>
+          <t>שכונת נווה יהושע</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -17038,18 +17038,18 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>גן סאנשיין</t>
+          <t>הבית של אורה</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>שכונת נווה יהושע</t>
+          <t>שכונת רמת שקמה</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -17068,12 +17068,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>הבית של אורה</t>
+          <t>גן הבית של אמא</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>שכונת רמת שקמה</t>
+          <t>שכונת אזור הבילויים</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -17086,7 +17086,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21">
@@ -17188,12 +17188,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>גן ישראל חינוך מאיר</t>
+          <t>הגן של אביה</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>שכונת קריית בורוכוב</t>
+          <t>שכונת תל גנים</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -17206,18 +17206,18 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>גן גפן</t>
+          <t>גן ישראל חינוך מאיר</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>שכונת מתחם נגבה</t>
+          <t>שכונת קריית בורוכוב</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -17230,18 +17230,18 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>גן הבית של אמא</t>
+          <t>גן גפן</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>שכונת אזור הבילויים</t>
+          <t>שכונת מתחם נגבה</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -17254,7 +17254,7 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="28">
@@ -17452,12 +17452,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>הגן של נתן</t>
+          <t>המשפחתון של סילביה</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>שכונת נווה יהושע</t>
+          <t>שכונת רמת עמידר</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -17470,7 +17470,7 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37">
@@ -17548,12 +17548,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>מעון מרום נווה</t>
+          <t>הגן של רבקה</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>שכונת מרום נווה</t>
+          <t>שכונת נחלת גנים</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -17566,18 +17566,18 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>גן רון לי</t>
+          <t>מעון מרום נווה</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>שכונת הלל</t>
+          <t>שכונת מרום נווה</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -17590,13 +17590,13 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>משפחתון וגן של חן</t>
+          <t>גן רון לי</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -17614,13 +17614,13 @@
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>אכא עמותה לקידום חינוך הוליסטי</t>
+          <t>משפחתון וגן של חן</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -17638,18 +17638,18 @@
         <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>גן סאנשיין הגפן</t>
+          <t>אכא עמותה לקידום חינוך הוליסטי</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>שכונת גפן</t>
+          <t>שכונת הלל</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -17662,7 +17662,7 @@
         <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="45">
@@ -17740,12 +17740,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>פנדה קלאב</t>
+          <t>גן סאנשיין הגפן</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>שכונת תל יהודה</t>
+          <t>שכונת גפן</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -17758,7 +17758,7 @@
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="49">
@@ -17788,12 +17788,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>מסיבת גן אצל תמי</t>
+          <t>פנדה קלאב</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>שכונת חשמונאים</t>
+          <t>שכונת תל יהודה</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -17806,18 +17806,18 @@
         <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>המשפחתון של סילביה</t>
+          <t>מסיבת גן אצל תמי</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>שכונת רמת עמידר</t>
+          <t>שכונת חשמונאים</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -17830,18 +17830,18 @@
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>גן פיצפונים</t>
+          <t>הגן של נתן</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>שכונת כפר אז''ר</t>
+          <t>שכונת נווה יהושע</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -17854,7 +17854,7 @@
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="53">
@@ -18028,12 +18028,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>חושחושים</t>
+          <t>גן פיצפונים</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>שכונת בן גוריון</t>
+          <t>שכונת כפר אז''ר</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -18046,7 +18046,7 @@
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61">
@@ -18124,12 +18124,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>גן תותי</t>
+          <t>חושחושים</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>שכונת מתחם נגבה</t>
+          <t>שכונת בן גוריון</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -18142,7 +18142,7 @@
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="65">
@@ -18220,12 +18220,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>גן מעון הנרקיסים</t>
+          <t>גן לאה</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>שכונת שיכון ותיקים</t>
+          <t>שכונת רמת עמידר</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -18238,7 +18238,7 @@
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="69">
@@ -18292,12 +18292,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>יהדות בחוויה</t>
+          <t>גן תותי</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>שכונת בן גוריון</t>
+          <t>שכונת מתחם נגבה</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -18310,7 +18310,7 @@
         <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="72">
@@ -18820,12 +18820,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>פשוש תל השומר</t>
+          <t>לה קסיטה דה צ'וקולטה</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>שכונת תל השומר</t>
+          <t>שכונת קריית בורוכוב</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -18838,18 +18838,18 @@
         <v>0</v>
       </c>
       <c r="F93" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>פעימות  רמת גן</t>
+          <t>פשוש תל השומר</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>שכונת קריית בורוכוב</t>
+          <t>שכונת תל השומר</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -18862,18 +18862,18 @@
         <v>0</v>
       </c>
       <c r="F94" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>גן פימפונים | פימפונים</t>
+          <t>פעימות  רמת גן</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>שכונת נווה רם</t>
+          <t>שכונת קריית בורוכוב</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -18886,18 +18886,18 @@
         <v>0</v>
       </c>
       <c r="F95" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>המשפחתון של שרון</t>
+          <t>גן פימפונים | פימפונים</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>שכונת גפן</t>
+          <t>שכונת נווה רם</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -18910,7 +18910,7 @@
         <v>0</v>
       </c>
       <c r="F96" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="97">
@@ -18940,7 +18940,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>המשפחתון של שרון ב</t>
+          <t>המשפחתון של שרון</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -18964,12 +18964,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>גן לאה</t>
+          <t>המשפחתון של שרון ב</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>שכונת רמת עמידר</t>
+          <t>שכונת גפן</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -18982,7 +18982,7 @@
         <v>0</v>
       </c>
       <c r="F99" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="100">
@@ -19060,12 +19060,12 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>דומיק</t>
+          <t>יהדות בחוויה</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>שכונת אזור הבילויים</t>
+          <t>שכונת בן גוריון</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -19078,18 +19078,18 @@
         <v>0</v>
       </c>
       <c r="F103" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>משפחתון מאירה</t>
+          <t>מעון אופק</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>שכונת תל יהודה</t>
+          <t>שכונת קריית קריניצי</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -19102,18 +19102,18 @@
         <v>0</v>
       </c>
       <c r="F104" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>מעון אופק</t>
+          <t>גן בתנועה</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>שכונת קריית קריניצי</t>
+          <t>שכונת שיכון ותיקים</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -19137,7 +19137,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>שכונת שיכון ותיקים</t>
+          <t>שכונת איצטדיון</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -19150,13 +19150,13 @@
         <v>0</v>
       </c>
       <c r="F106" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>גן בתנועה</t>
+          <t>יהדות בחוויה</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -19174,18 +19174,18 @@
         <v>0</v>
       </c>
       <c r="F107" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>יהדות בחוויה</t>
+          <t>גן כוכב</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>שכונת איצטדיון</t>
+          <t>שכונת מרכז העיר</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -19198,7 +19198,7 @@
         <v>0</v>
       </c>
       <c r="F108" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="109">
@@ -19276,12 +19276,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>גן כוכב</t>
+          <t>גן חלילית</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>שכונת מרכז העיר</t>
+          <t>שכונת איצטדיון</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -19294,7 +19294,7 @@
         <v>0</v>
       </c>
       <c r="F112" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="113">
@@ -19324,12 +19324,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>גן חלילית</t>
+          <t>פני פרלמן</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>שכונת איצטדיון</t>
+          <t>שכונת שיכון ותיקים</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -19342,13 +19342,13 @@
         <v>0</v>
       </c>
       <c r="F114" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>פני פרלמן</t>
+          <t>גן מעון הנרקיסים</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -19366,7 +19366,7 @@
         <v>0</v>
       </c>
       <c r="F115" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="116">
@@ -19444,12 +19444,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>גן אמנויות נילי</t>
+          <t>דומיק</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>שכונת מתחם נגבה</t>
+          <t>שכונת אזור הבילויים</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -19462,7 +19462,7 @@
         <v>0</v>
       </c>
       <c r="F119" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="120">
@@ -19636,36 +19636,36 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>הגן של רבקה</t>
+          <t>גן אמנויות נילי</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>שכונת נחלת גנים</t>
+          <t>שכונת מתחם נגבה</t>
         </is>
       </c>
       <c r="C127" t="n">
         <v>3</v>
       </c>
       <c r="D127" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E127" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F127" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>הגן של אביה</t>
+          <t>המשפחתון של עדינה</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>שכונת תל גנים</t>
+          <t>שכונת גפן</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -19678,18 +19678,18 @@
         <v>1</v>
       </c>
       <c r="F128" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>המשפחתון של עדינה</t>
+          <t>משפחתון מאירה</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>שכונת גפן</t>
+          <t>שכונת תל יהודה</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -19702,31 +19702,31 @@
         <v>1</v>
       </c>
       <c r="F129" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>לה קסיטה דה צ'וקולטה</t>
+          <t>שד ויצו שקמה ג</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>שכונת קריית בורוכוב</t>
+          <t>שכונת רמת שקמה</t>
         </is>
       </c>
       <c r="C130" t="n">
         <v>3</v>
       </c>
       <c r="D130" t="n">
+        <v>1</v>
+      </c>
+      <c r="E130" t="n">
         <v>2</v>
       </c>
-      <c r="E130" t="n">
-        <v>1</v>
-      </c>
       <c r="F130" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="131">

</xml_diff>